<commit_message>
Analyze case 2 gpu_sweep and bayesopt results
</commit_message>
<xml_diff>
--- a/solar_lumped/docs/parameters.xlsx
+++ b/solar_lumped/docs/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/clara/github-repos/SAWH_TEAs/solar_lumped/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DCA147-DADE-104B-AF49-B11585E248C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44B0692F-3E27-B542-B18B-7BBF1B6CFF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2235,7 +2235,7 @@
         <v>139</v>
       </c>
       <c r="C19" s="2">
-        <v>8</v>
+        <v>1.5</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>140</v>

</xml_diff>